<commit_message>
Parte 2 Reto #3: David Patacon - Correcion en Excel con historias de usuario
</commit_message>
<xml_diff>
--- a/Laboratorio-3-DOSW/docs/historias de usuario y atributos de calidad.xlsx
+++ b/Laboratorio-3-DOSW/docs/historias de usuario y atributos de calidad.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a11f14be0fe71ea4/2025-2/dosw/lab3 dosw/Labotatorio-3-DOSW/Laboratorio-3-DOSW/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aleja\OneDrive\Desktop\6 SEMESTRE\DOSW\PRIMER CORTE\LAB03\Labotatorio-3-DOSW\Laboratorio-3-DOSW\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="126" documentId="8_{2D6C90F7-E44C-4DAF-BBA2-A2252D3620A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06ADF86E-B93D-413F-96CB-3E62866C629E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B683F1C-70B4-4BB7-A47A-0D7CCF7ED617}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{8EDA342E-631D-40F7-A149-EBE673171BE5}"/>
+    <workbookView xWindow="-22524" yWindow="996" windowWidth="21600" windowHeight="11292" activeTab="3" xr2:uid="{8EDA342E-631D-40F7-A149-EBE673171BE5}"/>
   </bookViews>
   <sheets>
     <sheet name="cliente" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="21">
   <si>
     <t>Historia de Usuario</t>
   </si>
@@ -56,9 +56,6 @@
     <t>COMO cliente QUIERO depositar dinero en mi cuenta PARA PODER incrementar mi saldo y poder realizar futuras transacciones.</t>
   </si>
   <si>
-    <t xml:space="preserve">COMO cliente QUIERO ser notificado si mi saldo se vuelve negativo PARA PODER tomar acciones correctivas y regularizar mi estado financiero.    </t>
-  </si>
-  <si>
     <t>COMO administrador QUIERO registrar nuevos bancos en la lista de bancos autorizados y sus códigos PARA PODER ampliar nuestra oferta.</t>
   </si>
   <si>
@@ -72,9 +69,6 @@
   </si>
   <si>
     <t xml:space="preserve"> COMO sistema QUIERO rechazar cualquier depósito que tenga un monto negativo PARA PODER garantizar la lógica y la validez de las transacciones financieras.</t>
-  </si>
-  <si>
-    <t>COMO sistema QUIERO impedir una transferencia si la cuenta de origen no tiene saldo suficiente PARA PODER prevenir sobregiros no autorizados y mantener la solvencia del sistema.</t>
   </si>
   <si>
     <t>COMO desarrollador QUIERO que el código sea analizado automáticamente por SonarQube tras cada cambio PARA PODER identificar y corregir vulnerabilidades y problemas de calidad de manera proactiva.</t>
@@ -210,15 +204,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -248,7 +239,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -564,55 +555,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8637F09D-E0DB-4810-BB93-B1AC38A6DB3F}">
-  <dimension ref="B1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B1:C5"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="27.77734375" customWidth="1"/>
+    <col min="2" max="2" width="27.7109375" customWidth="1"/>
     <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="2:3" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+    </row>
+    <row r="3" spans="2:3" ht="82.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="2:3" ht="72" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" ht="90" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="2:3" ht="72" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" ht="90" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="2:3" ht="72" x14ac:dyDescent="0.3">
-      <c r="B6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -627,46 +610,46 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{184248D1-126B-4B00-A8D8-193A9B30F54B}">
   <dimension ref="B1:C5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.77734375" customWidth="1"/>
-    <col min="3" max="3" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" customWidth="1"/>
+    <col min="3" max="3" width="24.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="2:3" ht="85.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+    </row>
+    <row r="3" spans="2:3" ht="85.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" ht="106.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="2:3" ht="106.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" ht="165" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="2:3" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="B5" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="C5" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -680,47 +663,39 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9CBA1C6-093C-44A2-82D4-97A2B72509DD}">
-  <dimension ref="B1:C5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B1:C4"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="31.5546875" customWidth="1"/>
+    <col min="2" max="2" width="31.5703125" customWidth="1"/>
     <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="2:3" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+    </row>
+    <row r="3" spans="2:3" ht="105" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="2:3" ht="72" x14ac:dyDescent="0.3">
-      <c r="B4" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="C4" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="2:3" ht="72" x14ac:dyDescent="0.3">
-      <c r="B5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -735,38 +710,38 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{147A1F9C-62D9-4625-A898-8917D44F88A6}">
   <dimension ref="B1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="25.44140625" customWidth="1"/>
-    <col min="3" max="3" width="24.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.42578125" customWidth="1"/>
+    <col min="3" max="3" width="24.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B1" s="4" t="s">
+    <row r="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-    </row>
-    <row r="3" spans="2:3" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+    </row>
+    <row r="3" spans="2:3" ht="150" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="2:3" ht="144" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" ht="165" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>